<commit_message>
Fix(sunburst): omit empty objectives, clean cumplimiento_pct, export diagnostics; add logic docs
</commit_message>
<xml_diff>
--- a/artifacts/sunburst_diag_grouped.xlsx
+++ b/artifacts/sunburst_diag_grouped.xlsx
@@ -1,94 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
-  <si>
-    <t>Linea</t>
-  </si>
-  <si>
-    <t>Objetivo</t>
-  </si>
-  <si>
-    <t>cumplimiento_pct</t>
-  </si>
-  <si>
-    <t>Calidad</t>
-  </si>
-  <si>
-    <t>Educación_para_toda_la_vida</t>
-  </si>
-  <si>
-    <t>Expansión</t>
-  </si>
-  <si>
-    <t>Experiencia</t>
-  </si>
-  <si>
-    <t>Sostenibilidad</t>
-  </si>
-  <si>
-    <t>Transformación_Organizacional</t>
-  </si>
-  <si>
-    <t>Asegurar la alta calidad a nivel institucional</t>
-  </si>
-  <si>
-    <t>Fortalecer la oferta educativa y la innovación curricular</t>
-  </si>
-  <si>
-    <t>Impulsar y potenciar la educación continua</t>
-  </si>
-  <si>
-    <t>Crecer con compromiso social</t>
-  </si>
-  <si>
-    <t>Garantizar una experiencia significativa y de valor agregado a la comunidad POLI</t>
-  </si>
-  <si>
-    <t>Contribuir a la inclusión, la proyección social y el cuidado del medio ambiente</t>
-  </si>
-  <si>
-    <t>Promover una cultura de optimización de recursos financieros como apalancador de la estrategia</t>
-  </si>
-  <si>
-    <t>Asegurar una arquitectura tecnológica institucional, centrada en la experiencia de la comunidad educativa</t>
-  </si>
-  <si>
-    <t>Contar con un equipo humano feliz y apasionado, que trabaja de forma colaborativa para alcanzar las metas institucionales</t>
-  </si>
-  <si>
-    <t>Fortalecer la gestión por procesos y la toma de decisiones basada en el análisis de los datos</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -107,13 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -401,132 +408,182 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Objetivo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>cumplimiento_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Calidad</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Asegurar la alta calidad a nivel institucional</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>170.1950479917858</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Calidad</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fortalecer la oferta educativa y la innovación curricular</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>157.2715757883784</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Educación_para_toda_la_vida</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Impulsar y potenciar la educación continua</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>110.2612004693534</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Expansión</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Crecer con compromiso social</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>118.9224104645701</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Experiencia</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Garantizar una experiencia significativa y de valor agregado a la comunidad POLI</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>131.76620352111</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sostenibilidad</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Contribuir a la inclusión, la proyección social y el cuidado del medio ambiente</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>1801.124578480279</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sostenibilidad</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Promover una cultura de optimización de recursos financieros como apalancador de la estrategia</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>128.4317149971483</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Transformación_Organizacional</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Asegurar una arquitectura tecnológica institucional, centrada en la experiencia de la comunidad educativa</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>100.4049940236068</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Transformación_Organizacional</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Contar con un equipo humano feliz y apasionado, que trabaja de forma colaborativa para alcanzar las metas institucionales</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>409.1685256222597</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Transformación_Organizacional</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Fortalecer la gestión por procesos y la toma de decisiones basada en el análisis de los datos</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>127.3187606394003</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajustes codigo y visuales
</commit_message>
<xml_diff>
--- a/artifacts/sunburst_diag_grouped.xlsx
+++ b/artifacts/sunburst_diag_grouped.xlsx
@@ -424,7 +424,7 @@
         <v>9</v>
       </c>
       <c r="C2">
-        <v>110.183481573127</v>
+        <v>112.0501482397937</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -435,7 +435,7 @@
         <v>10</v>
       </c>
       <c r="C3">
-        <v>101.7416666666667</v>
+        <v>101.30625</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -446,7 +446,7 @@
         <v>11</v>
       </c>
       <c r="C4">
-        <v>108.89</v>
+        <v>108.8866587159206</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -457,7 +457,7 @@
         <v>12</v>
       </c>
       <c r="C5">
-        <v>113.0403624661247</v>
+        <v>108.4325377701309</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -468,7 +468,7 @@
         <v>13</v>
       </c>
       <c r="C6">
-        <v>104.6994700270681</v>
+        <v>104.6973696680775</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -479,7 +479,7 @@
         <v>14</v>
       </c>
       <c r="C7">
-        <v>104.1480072463768</v>
+        <v>103.8842918079195</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -490,7 +490,7 @@
         <v>15</v>
       </c>
       <c r="C8">
-        <v>118.2742989139818</v>
+        <v>116.4667608159802</v>
       </c>
     </row>
     <row r="9" spans="1:3">

</xml_diff>